<commit_message>
Add game 26-09-10_1: Capobranco/Pazzo win (Giovane Lupo wins via Branco, Lupo Reietto standalone excluded)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3031,7 +3031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI39"/>
+  <dimension ref="A1:AJ39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3216,6 +3216,11 @@
           <t>26-08-27_2</t>
         </is>
       </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>26-09-10_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3358,6 +3363,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3567,6 +3577,11 @@
           <t>Oste</t>
         </is>
       </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3875,6 +3890,11 @@
           <t>Oste</t>
         </is>
       </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4156,6 +4176,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Contadino</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4380,6 +4405,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4497,6 +4527,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4709,6 +4744,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Guardia Corrotta</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4801,6 +4841,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Sensitiva</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5032,6 +5077,11 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>Azzeccagarbugli</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5151,6 +5201,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5243,6 +5298,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5463,6 +5523,11 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5505,6 +5570,11 @@
       <c r="AI39" t="inlineStr">
         <is>
           <t>Assassino</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>Inquisitore</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5932,6 +6002,18 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>1 luna e 2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>26-09-10_1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Faida Inquisizione Sensitiva</t>
         </is>
       </c>
     </row>
@@ -5947,7 +6029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6323,6 +6405,18 @@
       <c r="B31" t="inlineStr">
         <is>
           <t>Prete custodito da Angelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>26-09-10_1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Angelo di Monaco; Monaco no Lupo del Branco no Vampiro, Contadino Lupo</t>
         </is>
       </c>
     </row>
@@ -6338,7 +6432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6916,6 +7010,23 @@
       <c r="C34" t="inlineStr">
         <is>
           <t>Capobranco Maledetto, Lupo del Branco</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>26-09-10_1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Capobranco, Pazzo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Giovane Lupo, Pazzo, Capobranco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-09-10_2: Villaggio/Mistici win (amanti lose), Fanatico=Giullare (via Giullare Modificato target), Prete=Romeo
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3031,7 +3031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ39"/>
+  <dimension ref="A1:AK39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3221,6 +3221,11 @@
           <t>26-09-10_1</t>
         </is>
       </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3368,6 +3373,11 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3582,6 +3592,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3895,6 +3910,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3957,6 +3977,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4181,6 +4206,11 @@
           <t>Contadino</t>
         </is>
       </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4410,6 +4440,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4532,6 +4567,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4749,6 +4789,11 @@
           <t>Guardia Corrotta</t>
         </is>
       </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4935,6 +4980,11 @@
           <t>Prete</t>
         </is>
       </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5082,6 +5132,11 @@
           <t>Azzeccagarbugli</t>
         </is>
       </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5206,6 +5261,11 @@
           <t>Pazzo</t>
         </is>
       </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>Bocca di Rosa</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5303,6 +5363,11 @@
           <t>Lupo Reietto</t>
         </is>
       </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>Borgomastro</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5528,6 +5593,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5575,6 +5645,11 @@
       <c r="AJ39" t="inlineStr">
         <is>
           <t>Inquisitore</t>
+        </is>
+      </c>
+      <c r="AK39" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
         </is>
       </c>
     </row>
@@ -5590,7 +5665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6014,6 +6089,18 @@
       <c r="B35" t="inlineStr">
         <is>
           <t>2 lune SÌ Faida Inquisizione Sensitiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Faida Fanatico Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6417,6 +6504,18 @@
       <c r="B32" t="inlineStr">
         <is>
           <t>Angelo di Monaco; Monaco no Lupo del Branco no Vampiro, Contadino Lupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Giulietta di Prete; Monaco no Eremita, Traditore, Strega, Guaritore</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7027,6 +7126,23 @@
       <c r="C35" t="inlineStr">
         <is>
           <t>Giovane Lupo, Pazzo, Capobranco</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Veggente, Bocca di Rosa, Borgomastro, Mago, Bardo, Monaco</t>
         </is>
       </c>
     </row>
@@ -7042,7 +7158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7504,6 +7620,40 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Lu'</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>albertasestito</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Romeo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 26-09-10_2: swap Rosario and Tullio's roles (Rosario=Lupo del Branco, Tullio=Veggente)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -4791,7 +4791,7 @@
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>Veggente</t>
+          <t>Lupo del Branco</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>Lupo del Branco</t>
+          <t>Veggente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix 26-08-05_2: win also includes Mistici, adding Rosario (Strega) and Massimo (Veggente) as winners
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -7069,12 +7069,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Villaggio, Angelo</t>
+          <t>Villaggio, Mistici, Angelo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Medium, Fanatico, Angelo</t>
+          <t>Medium, Fanatico, Angelo, Strega, Veggente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add players Krobbi, Garuni, Cacioppoli (Marco); add game 26-09-16_1: Lupo Solitario win (Traditore + Fanatico=Lupo Solitario), 3 winners
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -937,6 +937,42 @@
         </is>
       </c>
       <c r="B39" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Krobbi</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Krobbi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Garuni</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Garuni</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Cacioppoli</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>Marco</t>
         </is>
@@ -3031,7 +3067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK39"/>
+  <dimension ref="A1:AL42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3226,6 +3262,11 @@
           <t>26-09-10_2</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>26-09-16_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3378,6 +3419,11 @@
           <t>Giullare Modificato</t>
         </is>
       </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Traditore</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3915,6 +3961,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4084,6 +4135,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4211,6 +4267,11 @@
           <t>Prete</t>
         </is>
       </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4445,6 +4506,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4641,6 +4707,11 @@
           <t>Inquisitore</t>
         </is>
       </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>Spia</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5137,6 +5208,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>Lupo Solitario</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5266,6 +5342,11 @@
           <t>Bocca di Rosa</t>
         </is>
       </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5368,6 +5449,11 @@
           <t>Borgomastro</t>
         </is>
       </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>Sensitiva</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5598,6 +5684,11 @@
           <t>Lupo Reietto</t>
         </is>
       </c>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5650,6 +5741,57 @@
       <c r="AK39" t="inlineStr">
         <is>
           <t>Capobranco</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Krobbi</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Krobbi</t>
+        </is>
+      </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Garuni</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Garuni</t>
+        </is>
+      </c>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Cacioppoli</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>Prete</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6099,6 +6241,18 @@
         </is>
       </c>
       <c r="B36" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Faida Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>26-09-16_1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Faida Fanatico Giullare Modificato</t>
         </is>
@@ -6116,7 +6270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6516,6 +6670,18 @@
       <c r="B33" t="inlineStr">
         <is>
           <t>Giulietta di Prete; Monaco no Eremita, Traditore, Strega, Guaritore</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>26-09-16_1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Monaco no Villaggio, Mistici, Criminali, Inquisizione; Fanatico del Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -6531,7 +6697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7143,6 +7309,23 @@
       <c r="C36" t="inlineStr">
         <is>
           <t>Veggente, Bocca di Rosa, Borgomastro, Mago, Bardo, Monaco</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>26-09-16_1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Lupo Solitario</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Lupo Solitario, Fanatico, Traditore</t>
         </is>
       </c>
     </row>
@@ -7158,7 +7341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7654,6 +7837,23 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>26-09-16_1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>The Watcher</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 26-09-16_1: Marco Cacioppoli is Nulter, not a new player; remove erroneous Cacioppoli entry
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -963,18 +963,6 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>Garuni</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Cacioppoli</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Marco</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL42"/>
+  <dimension ref="A1:AL41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -5743,6 +5731,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5775,23 +5768,6 @@
       <c r="AL41" t="inlineStr">
         <is>
           <t>Giullare Modificato</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Cacioppoli</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
-      <c r="AL42" t="inlineStr">
-        <is>
-          <t>Prete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-09-16_2: Criminali win (Ladra only)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3055,7 +3055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL41"/>
+  <dimension ref="A1:AM41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3255,6 +3255,11 @@
           <t>26-09-16_1</t>
         </is>
       </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>26-09-16_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4021,6 +4026,11 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4499,6 +4509,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4700,6 +4715,11 @@
           <t>Spia</t>
         </is>
       </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4853,6 +4873,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5044,6 +5069,11 @@
           <t>Bardo</t>
         </is>
       </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5201,6 +5231,11 @@
           <t>Lupo Solitario</t>
         </is>
       </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5335,6 +5370,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5442,6 +5482,11 @@
           <t>Sensitiva</t>
         </is>
       </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>Ladra</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5751,6 +5796,11 @@
       <c r="AL40" t="inlineStr">
         <is>
           <t>Guardia</t>
+        </is>
+      </c>
+      <c r="AM40" t="inlineStr">
+        <is>
+          <t>Contadino</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6231,6 +6281,18 @@
       <c r="B37" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Faida Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>26-09-16_2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6673,7 +6735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7302,6 +7364,23 @@
       <c r="C37" t="inlineStr">
         <is>
           <t>Lupo Solitario, Fanatico, Traditore</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>26-09-16_2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Criminali</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ladra</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix 26-09-16_1: Prete was Marco (Tamburrino), not Nulter
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -5069,6 +5069,11 @@
           <t>Bardo</t>
         </is>
       </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
       <c r="AM23" t="inlineStr">
         <is>
           <t>Guardia</t>
@@ -5774,11 +5779,6 @@
       <c r="AK39" t="inlineStr">
         <is>
           <t>Capobranco</t>
-        </is>
-      </c>
-      <c r="AL39" t="inlineStr">
-        <is>
-          <t>Prete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-09-03_1: Villaggio win (Cacciatore di Vampiri, Eremita, Guardia, Contadino Lupo)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3055,7 +3055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM41"/>
+  <dimension ref="A1:AN41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3260,6 +3260,11 @@
           <t>26-09-16_2</t>
         </is>
       </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>26-09-03_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3417,6 +3422,11 @@
           <t>Traditore</t>
         </is>
       </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3479,6 +3489,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3842,6 +3857,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4138,6 +4158,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4514,6 +4539,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4878,6 +4908,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4975,6 +5010,11 @@
           <t>Sensitiva</t>
         </is>
       </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5079,6 +5119,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5241,6 +5286,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5380,6 +5430,11 @@
           <t>Bardo</t>
         </is>
       </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Contadino Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5779,6 +5834,11 @@
       <c r="AK39" t="inlineStr">
         <is>
           <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr">
+        <is>
+          <t>Eremita</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6293,6 +6353,18 @@
       <c r="B38" t="inlineStr">
         <is>
           <t>2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>26-09-03_1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico Maledizioni</t>
         </is>
       </c>
     </row>
@@ -6308,7 +6380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6720,6 +6792,18 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>Monaco no Villaggio, Mistici, Criminali, Inquisizione; Fanatico del Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>26-09-03_1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Angelo di Cacciatore di Vampiri</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7381,6 +7465,23 @@
       <c r="C38" t="inlineStr">
         <is>
           <t>Ladra</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>26-09-03_1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri, Eremita, Guardia, Contadino Lupo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-09-03_2: Villaggio win (Altra Guardia, Fanatico=Villaggio, Peccatore)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3055,7 +3055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN41"/>
+  <dimension ref="A1:AO41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3265,6 +3265,11 @@
           <t>26-09-03_1</t>
         </is>
       </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>26-09-03_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3427,6 +3432,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3494,6 +3504,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3862,6 +3877,11 @@
           <t>Negromante</t>
         </is>
       </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4163,6 +4183,11 @@
           <t>Vampiro</t>
         </is>
       </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4544,6 +4569,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4750,6 +4780,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4913,6 +4948,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>Guaritore</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5124,6 +5164,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5291,6 +5336,11 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5435,6 +5485,11 @@
           <t>Contadino Lupo</t>
         </is>
       </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>Peccatore</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5839,6 +5894,11 @@
       <c r="AN39" t="inlineStr">
         <is>
           <t>Eremita</t>
+        </is>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>Mago</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6365,6 +6425,18 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico Maledizioni</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>26-09-03_2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Faida Fanatico</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6804,6 +6876,18 @@
       <c r="B35" t="inlineStr">
         <is>
           <t>Angelo di Cacciatore di Vampiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>26-09-03_2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Fanatico dell'Altra Guardia</t>
         </is>
       </c>
     </row>
@@ -6819,7 +6903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7482,6 +7566,23 @@
       <c r="C39" t="inlineStr">
         <is>
           <t>Cacciatore di Vampiri, Eremita, Guardia, Contadino Lupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>26-09-03_2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Altra Guardia, Fanatico, Peccatore</t>
         </is>
       </c>
     </row>
@@ -7497,7 +7598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8010,6 +8111,23 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>26-09-03_2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Massimo</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-09-02_1: Criminali win (Guardia Corrotta only), Fanatico=Guaritore's Mistici
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3055,7 +3055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO41"/>
+  <dimension ref="A1:AP41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3270,6 +3270,11 @@
           <t>26-09-03_2</t>
         </is>
       </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>26-09-02_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3437,6 +3442,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>Guaritore</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3718,6 +3728,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3999,6 +4014,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4320,6 +4340,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4574,6 +4599,11 @@
           <t>Altra Guardia</t>
         </is>
       </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4701,6 +4731,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5169,6 +5204,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5341,6 +5381,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>Guardia Corrotta</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5490,6 +5535,11 @@
           <t>Peccatore</t>
         </is>
       </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5600,6 +5650,11 @@
       <c r="AM27" t="inlineStr">
         <is>
           <t>Ladra</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>Angelo</t>
         </is>
       </c>
     </row>
@@ -5953,7 +6008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6437,6 +6492,18 @@
       <c r="B40" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Faida Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>26-09-02_1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6888,6 +6955,18 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>Fanatico dell'Altra Guardia</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>26-09-02_1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Angelo di Fanatico; Fanatico del Guaritore</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7583,6 +7662,23 @@
       <c r="C40" t="inlineStr">
         <is>
           <t>Altra Guardia, Fanatico, Peccatore</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>26-09-02_1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Criminali</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Guardia Corrotta</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8128,6 +8224,23 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>26-09-02_1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>albertasestito</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Mistici</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add games.modalita (Discord/Live) tag, backfilled to Discord for all 40 existing games; show it in Composizione partita. Add 3 new Live games from 28 August: Criminali win, Capobranco/Pazzo win (Fanatico del Pazzo), Villaggio win (Tullio vampirizzato)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNotes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PWin" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POverrides" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PModalita" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Giocatori'!$A$1:$B$6</definedName>
@@ -457,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -963,6 +964,30 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>Garuni</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mattia</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Mattia</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sergio</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP41"/>
+  <dimension ref="A1:AS43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3275,6 +3300,21 @@
           <t>26-09-02_1</t>
         </is>
       </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>26-08-28_1</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>26-08-28_2</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3447,6 +3487,11 @@
           <t>Guaritore</t>
         </is>
       </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3897,6 +3942,21 @@
           <t>Giullare</t>
         </is>
       </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4019,6 +4079,21 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>Bocca di Rosa</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4604,6 +4679,21 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4736,6 +4826,16 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5090,6 +5190,21 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>Assassino</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5386,6 +5501,21 @@
           <t>Guardia Corrotta</t>
         </is>
       </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5713,6 +5843,21 @@
           <t>Prete</t>
         </is>
       </c>
+      <c r="AQ30" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="AR30" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5956,6 +6101,21 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AQ39" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>Contadino</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5993,6 +6153,60 @@
       <c r="AL41" t="inlineStr">
         <is>
           <t>Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mattia</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Mattia</t>
+        </is>
+      </c>
+      <c r="AQ42" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
+      <c r="AR42" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="AQ43" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
+      <c r="AR43" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>Eremita</t>
         </is>
       </c>
     </row>
@@ -6008,7 +6222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6504,6 +6718,42 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>26-08-28_1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>26-08-28_2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6967,6 +7217,42 @@
       <c r="B37" t="inlineStr">
         <is>
           <t>Angelo di Fanatico; Fanatico del Guaritore</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>26-08-28_1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Carte del Monaco: Capogilda, Ladra, Guaritore</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>26-08-28_2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Carte del Monaco: Guardia, Altra Guardia, Lupo del Branco</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Tullio (Giullare) è l'unico vampirizzato</t>
         </is>
       </c>
     </row>
@@ -6982,7 +7268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7679,6 +7965,57 @@
       <c r="C41" t="inlineStr">
         <is>
           <t>Guardia Corrotta</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>26-08-28_1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Criminali</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Assassino</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>26-08-28_2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Capobranco, Pazzo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Capobranco, Giovane Lupo, Fanatico, Pazzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri, Fanatico, Contadino, Eremita</t>
         </is>
       </c>
     </row>
@@ -7694,7 +8031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8241,6 +8578,616 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>26-08-28_1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Indo</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Romeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>26-08-28_2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Margherita</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TuBo97</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Anya</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>play</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>modalita</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>26-07-01_1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>26-07-01_2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>26-07-02_1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>26-07-02_2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>26-05-21_1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>26-06-03_1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>26-04-24_1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>26-06-25_1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>26-05-02_1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>26-06-03_2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>26-04-16_1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>26-05-29_1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>26-05-07_1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>26-05-14_1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>26-07-08_1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>26-07-08_2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>26-07-14_1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>26-07-14_2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>26-07-16_1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>26-07-16_2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>26-06-17_2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>26-07-23_2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>26-07-30_1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>26-07-30_2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26-08-21_1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>26-08-05_1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>26-08-11_1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>26-08-11_2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>26-08-21_2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>26-08-05_2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>26-08-27_1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>26-08-27_2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>26-09-10_1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>26-09-10_2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>26-09-16_1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>26-09-16_2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>26-09-03_1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>26-09-03_2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>26-09-02_1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>26-08-28_1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>26-08-28_2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>26-08-28_3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Apply rule: Villaggio win with no Inquisizione member present also credits Mistici. Fixed 26-07-08_2, 26-09-03_1, 26-09-03_2, 26-08-28_3
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Villaggio, Angelo</t>
+          <t>Villaggio, Angelo, Mistici</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -7925,12 +7925,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Villaggio</t>
+          <t>Villaggio, Mistici</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Cacciatore di Vampiri, Eremita, Guardia, Contadino Lupo</t>
+          <t>Cacciatore di Vampiri, Eremita, Guardia, Contadino Lupo, Veggente, Mago</t>
         </is>
       </c>
     </row>
@@ -7942,12 +7942,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Villaggio</t>
+          <t>Villaggio, Mistici</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Altra Guardia, Fanatico, Peccatore</t>
+          <t>Altra Guardia, Fanatico, Peccatore, Veggente, Mago, Guaritore</t>
         </is>
       </c>
     </row>
@@ -8010,12 +8010,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Villaggio</t>
+          <t>Villaggio, Mistici</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cacciatore di Vampiri, Fanatico, Contadino, Eremita</t>
+          <t>Cacciatore di Vampiri, Fanatico, Contadino, Eremita, Mago, Veggente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename all Discord games to 'Discord Live'; add game 26-09-18_1 (multi-day, 14-18 Sept) tagged 'Discord in-real time': Criminali/Città win
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS43"/>
+  <dimension ref="A1:AT43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3315,6 +3315,11 @@
           <t>26-08-28_3</t>
         </is>
       </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>26-09-18_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3492,6 +3497,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Sensitiva</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3721,6 +3731,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>Azzeccagarbugli</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3957,6 +3972,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4094,6 +4114,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4166,6 +4191,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4283,6 +4313,11 @@
           <t>Lupo Reietto</t>
         </is>
       </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4420,6 +4455,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4694,6 +4734,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4836,6 +4881,11 @@
           <t>Vampiro</t>
         </is>
       </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>Traditore</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5088,6 +5138,11 @@
           <t>Guaritore</t>
         </is>
       </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5205,6 +5260,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>Capogilda</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5262,6 +5322,11 @@
           <t>Ladra</t>
         </is>
       </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5324,6 +5389,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5514,6 +5584,11 @@
       <c r="AS24" t="inlineStr">
         <is>
           <t>Giullare</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>MASTER</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6754,6 +6829,18 @@
       <c r="B44" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>26-09-18_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare</t>
         </is>
       </c>
     </row>
@@ -6769,7 +6856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7253,6 +7340,18 @@
       <c r="B40" t="inlineStr">
         <is>
           <t>Tullio (Giullare) è l'unico vampirizzato</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>26-09-18_1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Partita durata dal 14 al 18 settembre 2026; Maledizioni (Negromante) su Dario e Filippo; Sensitiva gildata</t>
         </is>
       </c>
     </row>
@@ -7268,7 +7367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8016,6 +8115,23 @@
       <c r="C44" t="inlineStr">
         <is>
           <t>Cacciatore di Vampiri, Fanatico, Contadino, Eremita, Mago, Veggente</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>26-09-18_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Criminali, Città</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Capogilda, Sensitiva, Azzeccagarbugli, Mercante</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8643,6 +8759,23 @@
       <c r="C36" t="inlineStr">
         <is>
           <t>Villaggio</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>26-09-18_1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Massimo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Criminali</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8680,7 +8813,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8692,7 +8825,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8704,7 +8837,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8716,7 +8849,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8728,7 +8861,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8873,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8752,7 +8885,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8897,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8776,7 +8909,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8921,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8933,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8812,7 +8945,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8957,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8836,7 +8969,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8848,7 +8981,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8860,7 +8993,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8872,7 +9005,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8884,7 +9017,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8896,7 +9029,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8908,7 +9041,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8920,7 +9053,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8932,7 +9065,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8944,7 +9077,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8956,7 +9089,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8968,7 +9101,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8980,7 +9113,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -8992,7 +9125,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9137,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9016,7 +9149,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9028,7 +9161,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9040,7 +9173,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9052,7 +9185,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9064,7 +9197,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9076,7 +9209,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9088,7 +9221,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9233,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9112,7 +9245,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9124,7 +9257,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9269,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9148,7 +9281,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Discord</t>
+          <t>Discord Live</t>
         </is>
       </c>
     </row>
@@ -9185,6 +9318,18 @@
       <c r="B44" t="inlineStr">
         <is>
           <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>26-09-18_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Discord in-real time</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruoli Possibili: add commas between items within NO/SÌ clauses (not before the keyword); fix 26-08-27_1/_2 '1 luna e 2 lune' artifact to plain '2 lune'
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -6324,7 +6324,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Strega</t>
+          <t>2 lune NO Giullare, Strega</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Strega</t>
+          <t>2 lune NO Giullare, Strega</t>
         </is>
       </c>
     </row>
@@ -6420,7 +6420,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Vampiri</t>
+          <t>2 lune NO Giullare, Vampiri</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Vampiri SÌ Faida Fanatico</t>
+          <t>2 lune NO Giullare, Vampiri SÌ Faida, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6468,7 +6468,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Vampiri</t>
+          <t>2 lune NO Giullare, Vampiri</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Vampiri</t>
+          <t>2 lune NO Giullare, Vampiri</t>
         </is>
       </c>
     </row>
@@ -6504,7 +6504,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare SÌ Lupo Reietto Lupo Solitario</t>
+          <t>2 lune NO Giullare SÌ Lupo Reietto, Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6516,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare Amanti SÌ Faida Inquisizione Megera</t>
+          <t>2 lune NO Giullare, Amanti SÌ Faida, Inquisizione, Megera</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare SÌ Fanatico Sensitiva</t>
+          <t>2 lune NO Giullare SÌ Fanatico, Sensitiva</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare SÌ Fanatico Sensitiva</t>
+          <t>2 lune NO Giullare SÌ Fanatico, Sensitiva</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6576,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Giullare Modificato Negromante</t>
+          <t>2 lune SÌ Capobranco Maledetto, Giullare Modificato, Negromante</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare SÌ Inquisizione Megera</t>
+          <t>2 lune NO Giullare SÌ Inquisizione, Megera</t>
         </is>
       </c>
     </row>
@@ -6612,7 +6612,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Giullare Modificato</t>
+          <t>2 lune SÌ Capobranco Maledetto, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6624,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2 lune SÌ Faida Inquisizione</t>
+          <t>2 lune SÌ Faida, Inquisizione</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1 luna e 2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+          <t>2 lune NO Giullare SÌ Capobranco Maledetto, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1 luna e 2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+          <t>2 lune NO Giullare SÌ Capobranco Maledetto, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2 lune SÌ Faida Inquisizione Sensitiva</t>
+          <t>2 lune SÌ Faida, Inquisizione, Sensitiva</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Faida Fanatico Giullare Modificato</t>
+          <t>2 lune SÌ Capobranco Maledetto, Faida, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Faida Fanatico Giullare Modificato</t>
+          <t>2 lune SÌ Capobranco Maledetto, Faida, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+          <t>2 lune NO Giullare SÌ Capobranco Maledetto, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6768,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico Maledizioni</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico, Maledizioni</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Faida Fanatico</t>
+          <t>2 lune SÌ Capobranco Maledetto, Faida, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2 lune SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+          <t>2 lune SÌ Capobranco Maledetto, Fanatico, Giullare Modificato</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename player nick ZicNick -> ZicNik
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -821,7 +821,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ZicNick</t>
+          <t>ZicNik</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5749,7 +5749,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ZicNick</t>
+          <t>ZicNik</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>

<commit_message>
Add game 26-09-24_1 (Discord Live)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT43"/>
+  <dimension ref="A1:AU43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3320,6 +3320,11 @@
           <t>26-09-18_1</t>
         </is>
       </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>26-09-24_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3502,6 +3507,11 @@
           <t>Sensitiva</t>
         </is>
       </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3736,6 +3746,11 @@
           <t>Azzeccagarbugli</t>
         </is>
       </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4318,6 +4333,11 @@
           <t>Altra Guardia</t>
         </is>
       </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4460,6 +4480,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4739,6 +4764,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4886,6 +4916,11 @@
           <t>Traditore</t>
         </is>
       </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5143,6 +5178,11 @@
           <t>Negromante</t>
         </is>
       </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5265,6 +5305,11 @@
           <t>Capogilda</t>
         </is>
       </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5745,6 +5790,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5862,6 +5912,11 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6189,6 +6244,11 @@
       <c r="AS39" t="inlineStr">
         <is>
           <t>Contadino</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>Guardia</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6841,6 +6901,18 @@
       <c r="B45" t="inlineStr">
         <is>
           <t>2 lune NO Giullare</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>26-09-24_1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Becchino, Capobranco Maledetto, Giullare Modificato, Megera, Negromante</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7352,6 +7424,18 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>Partita durata dal 14 al 18 settembre 2026; Maledizioni (Negromante) su Dario e Filippo; Sensitiva gildata</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>26-09-24_1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Giulietta di Guardia; Monaco no Capobranco, Peccatore, Borgomastro; Maledetti (Capobranco Maledetto): Giullare Modificato e Medium</t>
         </is>
       </c>
     </row>
@@ -7367,7 +7451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8132,6 +8216,23 @@
       <c r="C45" t="inlineStr">
         <is>
           <t>Capogilda, Sensitiva, Azzeccagarbugli, Mercante</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>26-09-24_1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Capobranco, Giullare</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto, Lupo del Branco, Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8776,6 +8877,23 @@
       <c r="C37" t="inlineStr">
         <is>
           <t>Criminali</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>26-09-24_1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Nulter</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Romeo</t>
         </is>
       </c>
     </row>
@@ -8790,7 +8908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9333,6 +9451,18 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>26-09-24_1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-08_1 (Discord Live)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU43"/>
+  <dimension ref="A1:AV43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3325,6 +3325,11 @@
           <t>26-09-24_1</t>
         </is>
       </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>26-10-08_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3751,6 +3756,11 @@
           <t>Giullare Modificato</t>
         </is>
       </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3808,6 +3818,11 @@
           <t>Giullare</t>
         </is>
       </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4485,6 +4500,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4769,6 +4789,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5005,6 +5030,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5183,6 +5213,11 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5636,6 +5671,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5917,6 +5957,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6251,6 +6296,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>Bracconiere</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6273,6 +6323,11 @@
           <t>Contadino</t>
         </is>
       </c>
+      <c r="AV40" t="inlineStr">
+        <is>
+          <t>Guaritore</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6288,6 +6343,11 @@
       <c r="AL41" t="inlineStr">
         <is>
           <t>Giullare Modificato</t>
+        </is>
+      </c>
+      <c r="AV41" t="inlineStr">
+        <is>
+          <t>Mercante</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6913,6 +6973,18 @@
       <c r="B46" t="inlineStr">
         <is>
           <t>2 lune SÌ Becchino, Capobranco Maledetto, Giullare Modificato, Megera, Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>26-10-08_1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -6928,7 +7000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7436,6 +7508,18 @@
       <c r="B42" t="inlineStr">
         <is>
           <t>Giulietta di Guardia; Monaco no Capobranco, Peccatore, Borgomastro; Maledetti (Capobranco Maledetto): Giullare Modificato e Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>26-10-08_1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Fanatico del Medium; Maledizioni (Negromante) su ZicNik e Filippo</t>
         </is>
       </c>
     </row>
@@ -7451,7 +7535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8233,6 +8317,23 @@
       <c r="C46" t="inlineStr">
         <is>
           <t>Capobranco Maledetto, Lupo del Branco, Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>26-10-08_1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Negromante</t>
         </is>
       </c>
     </row>
@@ -8248,7 +8349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8894,6 +8995,23 @@
       <c r="C38" t="inlineStr">
         <is>
           <t>Romeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>26-10-08_1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
         </is>
       </c>
     </row>
@@ -8908,7 +9026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9463,6 +9581,18 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>26-10-08_1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-01_1 (Discord Live); display name MarcoC for nick Nulter
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -939,7 +939,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Marco</t>
+          <t>MarcoC</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV43"/>
+  <dimension ref="A1:AW43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3330,6 +3330,11 @@
           <t>26-10-08_1</t>
         </is>
       </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>26-10-01_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3517,6 +3522,11 @@
           <t>Negromante</t>
         </is>
       </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3589,6 +3599,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4353,6 +4368,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4505,6 +4525,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4794,6 +4819,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>Spia</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4946,6 +4976,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5218,6 +5253,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5345,6 +5385,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5474,6 +5519,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>Boia</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5835,6 +5885,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AW26" t="inlineStr">
+        <is>
+          <t>Inquisitore</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6243,7 +6298,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nulter (Marco)</t>
+          <t>Nulter (MarcoC)</t>
         </is>
       </c>
       <c r="AH39" t="inlineStr">
@@ -6299,6 +6354,11 @@
       <c r="AV39" t="inlineStr">
         <is>
           <t>Bracconiere</t>
+        </is>
+      </c>
+      <c r="AW39" t="inlineStr">
+        <is>
+          <t>Guardia</t>
         </is>
       </c>
     </row>
@@ -6417,7 +6477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6985,6 +7045,18 @@
       <c r="B47" t="inlineStr">
         <is>
           <t>2 lune SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>26-10-01_1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare SÌ Boia, Capobranco Maledetto, Fanatico, Giullare Modificato, Inquisitore</t>
         </is>
       </c>
     </row>
@@ -7000,7 +7072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7520,6 +7592,18 @@
       <c r="B43" t="inlineStr">
         <is>
           <t>Fanatico del Medium; Maledizioni (Negromante) su ZicNik e Filippo</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>26-10-01_1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Fanatico della Strega</t>
         </is>
       </c>
     </row>
@@ -7535,7 +7619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8334,6 +8418,23 @@
       <c r="C47" t="inlineStr">
         <is>
           <t>Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>26-10-01_1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Guardia, Eremita, Veggente, Strega, Fanatico</t>
         </is>
       </c>
     </row>
@@ -8349,7 +8450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9012,6 +9113,23 @@
       <c r="C39" t="inlineStr">
         <is>
           <t>Villaggio</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>26-10-01_1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Lu'</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mistici</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9593,6 +9711,18 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>26-10-01_1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-09-24_2 (Discord Live)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW43"/>
+  <dimension ref="A1:AX43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3335,6 +3335,11 @@
           <t>26-10-01_1</t>
         </is>
       </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>26-09-24_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3527,6 +3532,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3776,6 +3786,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4373,6 +4388,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4530,6 +4550,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4824,6 +4849,11 @@
           <t>Spia</t>
         </is>
       </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4981,6 +5011,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5070,6 +5105,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>Traditore</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5258,6 +5298,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>Bracconiere</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5726,6 +5771,11 @@
           <t>Negromante</t>
         </is>
       </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5763,6 +5813,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5890,6 +5945,11 @@
           <t>Inquisitore</t>
         </is>
       </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6015,6 +6075,11 @@
       <c r="AV27" t="inlineStr">
         <is>
           <t>Giovane Lupo</t>
+        </is>
+      </c>
+      <c r="AX27" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7057,6 +7122,18 @@
       <c r="B48" t="inlineStr">
         <is>
           <t>2 lune NO Giullare SÌ Boia, Capobranco Maledetto, Fanatico, Giullare Modificato, Inquisitore</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>26-09-24_2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Bracconiere, Lupo Reietto, Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7604,6 +7681,18 @@
       <c r="B44" t="inlineStr">
         <is>
           <t>Fanatico della Strega</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>26-09-24_2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Giulietta di Eremita; Monaco no Guardia, Pazzo, Giovane Lupo</t>
         </is>
       </c>
     </row>
@@ -7619,7 +7708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8435,6 +8524,23 @@
       <c r="C48" t="inlineStr">
         <is>
           <t>Guardia, Eremita, Veggente, Strega, Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>26-09-24_2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Veggente, Mago, Monaco, Medium, Bracconiere</t>
         </is>
       </c>
     </row>
@@ -8450,7 +8556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9130,6 +9236,23 @@
       <c r="C40" t="inlineStr">
         <is>
           <t>Mistici</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>26-09-24_2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Massimo</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Romeo</t>
         </is>
       </c>
     </row>
@@ -9144,7 +9267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9723,6 +9846,18 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>26-09-24_2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-08_2 (Discord Live)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX43"/>
+  <dimension ref="A1:AY43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3340,6 +3340,11 @@
           <t>26-09-24_2</t>
         </is>
       </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>26-10-08_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3791,6 +3796,11 @@
           <t>Lupo Reietto</t>
         </is>
       </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>Traditore</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4555,6 +4565,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4854,6 +4869,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5110,6 +5130,11 @@
           <t>Traditore</t>
         </is>
       </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5303,6 +5328,11 @@
           <t>Bracconiere</t>
         </is>
       </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>Oste</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5569,6 +5599,11 @@
           <t>Boia</t>
         </is>
       </c>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>Bocca di Rosa</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5776,6 +5811,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5950,6 +5990,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6082,6 +6127,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AY27" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6426,6 +6476,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AY39" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6451,6 +6506,11 @@
       <c r="AV40" t="inlineStr">
         <is>
           <t>Guaritore</t>
+        </is>
+      </c>
+      <c r="AY40" t="inlineStr">
+        <is>
+          <t>Guardia</t>
         </is>
       </c>
     </row>
@@ -6542,7 +6602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7134,6 +7194,18 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>2 lune SÌ Bracconiere, Lupo Reietto, Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>26-10-08_2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7693,6 +7765,18 @@
       <c r="B45" t="inlineStr">
         <is>
           <t>Giulietta di Eremita; Monaco no Guardia, Pazzo, Giovane Lupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>26-10-08_2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Fanatico del Traditore</t>
         </is>
       </c>
     </row>
@@ -7708,7 +7792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8541,6 +8625,23 @@
       <c r="C49" t="inlineStr">
         <is>
           <t>Veggente, Mago, Monaco, Medium, Bracconiere</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>26-10-08_2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Capobranco, Lupo del Branco, Traditore, Fanatico</t>
         </is>
       </c>
     </row>
@@ -8556,7 +8657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9253,6 +9354,23 @@
       <c r="C41" t="inlineStr">
         <is>
           <t>Romeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>26-10-08_2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Giuseppe</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Capobranco, Lupo Reietto, Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -9267,7 +9385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9858,6 +9976,18 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>26-10-08_2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-15_1 (Discord Live), new players Vincenzo and Johnny
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -988,6 +988,30 @@
       <c r="B43" t="inlineStr">
         <is>
           <t>Sergio</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Vincenzo</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Vincenzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Johnny</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Giovanni</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY43"/>
+  <dimension ref="A1:AZ45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3345,6 +3369,11 @@
           <t>26-10-08_2</t>
         </is>
       </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>26-10-15_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3863,6 +3892,11 @@
           <t>Lupo Reietto</t>
         </is>
       </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4189,6 +4223,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4266,6 +4305,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4570,6 +4614,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4874,6 +4923,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5333,6 +5387,11 @@
           <t>Oste</t>
         </is>
       </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5465,6 +5524,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>Borgomastro</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6132,6 +6196,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AZ27" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6513,6 +6582,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AZ40" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6562,6 +6636,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AZ42" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6587,6 +6666,40 @@
       <c r="AS43" t="inlineStr">
         <is>
           <t>Eremita</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Vincenzo</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Vincenzo</t>
+        </is>
+      </c>
+      <c r="AZ44" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Johnny</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Giovanni</t>
+        </is>
+      </c>
+      <c r="AZ45" t="inlineStr">
+        <is>
+          <t>Veggente</t>
         </is>
       </c>
     </row>
@@ -6602,7 +6715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7206,6 +7319,18 @@
       <c r="B50" t="inlineStr">
         <is>
           <t>2 lune SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>26-10-15_1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario, Negromante</t>
         </is>
       </c>
     </row>
@@ -7221,7 +7346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7777,6 +7902,18 @@
       <c r="B46" t="inlineStr">
         <is>
           <t>Fanatico del Traditore</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>26-10-15_1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Monaco no Altra Guardia, Guardia, Medium, Traditore; Fanatico del Borgomastro; Angelo del Borgomastro</t>
         </is>
       </c>
     </row>
@@ -7792,7 +7929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8642,6 +8779,23 @@
       <c r="C50" t="inlineStr">
         <is>
           <t>Capobranco, Lupo del Branco, Traditore, Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>26-10-15_1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto, Lupo del Branco, Giovane Lupo</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9371,6 +9525,23 @@
       <c r="C42" t="inlineStr">
         <is>
           <t>Capobranco, Lupo Reietto, Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>26-10-15_1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>albertasestito</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici, Criminali, Inquisizione</t>
         </is>
       </c>
     </row>
@@ -9385,7 +9556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9988,6 +10159,18 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>26-10-15_1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-15_2 (Discord Live)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3104,7 +3104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ45"/>
+  <dimension ref="A1:BA45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3374,6 +3374,11 @@
           <t>26-10-15_1</t>
         </is>
       </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>26-10-15_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3571,6 +3576,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4928,6 +4938,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5392,6 +5407,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6059,6 +6079,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="BA26" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6201,6 +6226,11 @@
           <t>Negromante</t>
         </is>
       </c>
+      <c r="BA27" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6550,6 +6580,11 @@
           <t>Bardo</t>
         </is>
       </c>
+      <c r="BA39" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6641,6 +6676,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="BA42" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6700,6 +6740,11 @@
       <c r="AZ45" t="inlineStr">
         <is>
           <t>Veggente</t>
+        </is>
+      </c>
+      <c r="BA45" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
         </is>
       </c>
     </row>
@@ -6715,7 +6760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7329,6 +7374,18 @@
         </is>
       </c>
       <c r="B51" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario, Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>26-10-15_2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario, Negromante</t>
         </is>
@@ -7346,7 +7403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7914,6 +7971,18 @@
       <c r="B47" t="inlineStr">
         <is>
           <t>Monaco no Altra Guardia, Guardia, Medium, Traditore; Fanatico del Borgomastro; Angelo del Borgomastro</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>26-10-15_2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Monaco no Azzeccagarbugli, Bardo, Oratore, Oste</t>
         </is>
       </c>
     </row>
@@ -7929,7 +7998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8796,6 +8865,23 @@
       <c r="C51" t="inlineStr">
         <is>
           <t>Capobranco Maledetto, Lupo del Branco, Giovane Lupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>26-10-15_2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Capobranco, Lupo del Branco</t>
         </is>
       </c>
     </row>
@@ -9556,7 +9642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10171,6 +10257,18 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>26-10-15_2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-22_1 (Discord Live)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3104,7 +3104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA45"/>
+  <dimension ref="A1:BB45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3379,6 +3379,11 @@
           <t>26-10-15_2</t>
         </is>
       </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3840,6 +3845,11 @@
           <t>Traditore</t>
         </is>
       </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4238,6 +4248,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4943,6 +4958,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5105,6 +5125,11 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5204,6 +5229,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>Peccatore</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5412,6 +5442,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5549,6 +5584,11 @@
           <t>Borgomastro</t>
         </is>
       </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>Borgomastro</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6231,6 +6271,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="BB27" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6585,6 +6630,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="BB39" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6622,6 +6672,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="BB40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6644,6 +6699,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="BB41" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6681,6 +6741,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="BB42" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6743,6 +6808,11 @@
         </is>
       </c>
       <c r="BA45" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="BB45" t="inlineStr">
         <is>
           <t>Capobranco</t>
         </is>
@@ -6760,7 +6830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7386,6 +7456,18 @@
         </is>
       </c>
       <c r="B52" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario, Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario, Negromante</t>
         </is>
@@ -7403,7 +7485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7983,6 +8065,18 @@
       <c r="B48" t="inlineStr">
         <is>
           <t>Monaco no Azzeccagarbugli, Bardo, Oratore, Oste</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Monaco no Negromante, Strega, Guaritore; Borgomastro e Peccatore vampirizzati</t>
         </is>
       </c>
     </row>
@@ -7998,7 +8092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8882,6 +8976,23 @@
       <c r="C52" t="inlineStr">
         <is>
           <t>Capobranco, Lupo del Branco</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Vampiro, Borgomastro, Peccatore</t>
         </is>
       </c>
     </row>
@@ -8897,7 +9008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9628,6 +9739,40 @@
       <c r="C43" t="inlineStr">
         <is>
           <t>Villaggio, Mistici, Criminali, Inquisizione</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>alfred8136</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>JoeHudson94</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
         </is>
       </c>
     </row>
@@ -9642,7 +9787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10269,6 +10414,18 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>26-10-22_1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-10-22_2 (Discord Live)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3104,7 +3104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB45"/>
+  <dimension ref="A1:BC45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3384,6 +3384,11 @@
           <t>26-10-22_1</t>
         </is>
       </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>26-10-22_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3850,6 +3855,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4253,6 +4263,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>Azzeccagarbugli</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4963,6 +4978,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5130,6 +5150,11 @@
           <t>Prete</t>
         </is>
       </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5234,6 +5259,11 @@
           <t>Peccatore</t>
         </is>
       </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5447,6 +5477,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5728,6 +5763,11 @@
           <t>Bocca di Rosa</t>
         </is>
       </c>
+      <c r="BC23" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6124,6 +6164,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="BC26" t="inlineStr">
+        <is>
+          <t>Assassino</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6276,6 +6321,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="BC27" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6635,6 +6685,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="BC39" t="inlineStr">
+        <is>
+          <t>Capogilda</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6677,6 +6732,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="BC40" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6704,6 +6764,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="BC41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6815,6 +6880,11 @@
       <c r="BB45" t="inlineStr">
         <is>
           <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="BC45" t="inlineStr">
+        <is>
+          <t>Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7470,6 +7540,18 @@
       <c r="B53" t="inlineStr">
         <is>
           <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario, Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>26-10-22_2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare SÌ Bracconiere, Capobranco Maledetto, Fanatico, Giullare Modificato, Lupo Reietto, Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8077,6 +8159,18 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>Monaco no Negromante, Strega, Guaritore; Borgomastro e Peccatore vampirizzati</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>26-10-22_2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Angelo di Altra Guardia; Medium gildato; Monaco no Eremita, Vampiro</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8993,6 +9087,23 @@
       <c r="C53" t="inlineStr">
         <is>
           <t>Vampiro, Borgomastro, Peccatore</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>26-10-22_2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici, Città, Angelo</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Guardia, Altra Guardia, Monaco, Veggente, Azzeccagarbugli, Angelo</t>
         </is>
       </c>
     </row>
@@ -9008,7 +9119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9773,6 +9884,23 @@
       <c r="C45" t="inlineStr">
         <is>
           <t>Vampiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>26-10-22_2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Garuni</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Criminali</t>
         </is>
       </c>
     </row>
@@ -9787,7 +9915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10426,6 +10554,18 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>26-10-22_2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Discord Live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Split Mattia Trama into a separate player from Mattia
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -1012,6 +1012,18 @@
       <c r="B45" t="inlineStr">
         <is>
           <t>Giovanni</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mattia Trama</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Mattia Trama</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC45"/>
+  <dimension ref="A1:BC46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -6885,6 +6897,33 @@
       <c r="BC45" t="inlineStr">
         <is>
           <t>Lupo Solitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mattia Trama</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Mattia Trama</t>
+        </is>
+      </c>
+      <c r="AZ46" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
+      <c r="BA46" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="BB46" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Mattia split: clear moved games from old Mattia row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -6808,21 +6808,6 @@
           <t>Mago</t>
         </is>
       </c>
-      <c r="AZ42" t="inlineStr">
-        <is>
-          <t>Capobranco Maledetto</t>
-        </is>
-      </c>
-      <c r="BA42" t="inlineStr">
-        <is>
-          <t>Monaco</t>
-        </is>
-      </c>
-      <c r="BB42" t="inlineStr">
-        <is>
-          <t>Vampiro</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">

</xml_diff>

<commit_message>
Rename Mattia Trama to nick Trama (nome Mattia); remove unused players
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -653,377 +653,353 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gianlu</t>
+          <t>JoeHudson94</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gianluca</t>
+          <t>GiorgioB</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>JoeHudson94</t>
+          <t>Ilaria</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GiorgioB</t>
+          <t>Ilaria</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ilaria</t>
+          <t>Lu'</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ilaria</t>
+          <t>Luca</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lu'</t>
+          <t>Marco</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Marco</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Marco</t>
+          <t>Margherita</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Marco</t>
+          <t>Margherita</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Margherita</t>
+          <t>Massimo</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Margherita</t>
+          <t>Massimo</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Massimo</t>
+          <t>CarMa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Massimo</t>
+          <t>Maurizio</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CarMa</t>
+          <t>rasel</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Maurizio</t>
+          <t>Pietro</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>rasel</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pietro</t>
+          <t>Rosario</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Anya</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Stefania</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Anya</t>
+          <t>TuBo97</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Stefania</t>
+          <t>Tullio</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TuBo97</t>
+          <t>sgargi</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tullio</t>
+          <t>Valerio</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sgargi</t>
+          <t>Giuseppe</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Valerio</t>
+          <t>Giuseppe</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Giuseppe</t>
+          <t>ZicNik</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Giuseppe</t>
+          <t>Giorgio</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ZicNik</t>
+          <t>AntonioL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Giorgio</t>
+          <t>Antonio</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>chani_kynes</t>
+          <t>Pasquale</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Simona</t>
+          <t>Pasquale</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AntonioL</t>
+          <t>Emanuele</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Antonio</t>
+          <t>Emanuele</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pasquale</t>
+          <t>er_divino</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pasquale</t>
+          <t>Simone</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Emanuele</t>
+          <t>Elena</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Emanuele</t>
+          <t>Elena</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>er_divino</t>
+          <t>Andrea</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lippo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Elena</t>
+          <t>Alessio</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Elena</t>
+          <t>Alessio</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Andrea</t>
+          <t>Nulter</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Andrea</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Lippo</t>
+          <t>MarcoC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alessio</t>
+          <t>Krobbi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alessio</t>
+          <t>Krobbi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Nulter</t>
+          <t>Garuni</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MarcoC</t>
+          <t>Garuni</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Krobbi</t>
+          <t>Mattia</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Krobbi</t>
+          <t>Mattia</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Garuni</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Garuni</t>
+          <t>Sergio</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mattia</t>
+          <t>Vincenzo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mattia</t>
+          <t>Vincenzo</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Johnny</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Giovanni</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vincenzo</t>
+          <t>Trama</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vincenzo</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Johnny</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Giovanni</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Mattia Trama</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Mattia Trama</t>
+          <t>Mattia</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC46"/>
+  <dimension ref="A1:BC44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -6413,397 +6389,417 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gianlu</t>
+          <t>Pasquale</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gianluca</t>
+          <t>Pasquale</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Mercante</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>chani_kynes</t>
+          <t>Emanuele</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Simona</t>
+          <t>Emanuele</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>Veggente</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pasquale</t>
+          <t>er_divino</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pasquale</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Mercante</t>
+          <t>Simone</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Bocca di Rosa</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>Capogilda</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Guardia</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Emanuele</t>
+          <t>Elena</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Emanuele</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>Capobranco</t>
+          <t>Elena</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Megera</t>
         </is>
       </c>
       <c r="AE34" t="inlineStr">
         <is>
-          <t>Veggente</t>
+          <t>Oste</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>er_divino</t>
+          <t>Andrea</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Simone</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>Oratore</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>Lupo Reietto</t>
+        </is>
+      </c>
+      <c r="AL35" t="inlineStr">
         <is>
           <t>Strega</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>Bocca di Rosa</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>Capogilda</t>
-        </is>
-      </c>
-      <c r="Y35" t="inlineStr">
-        <is>
-          <t>Veggente</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>Guardia</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Elena</t>
+          <t>Alessio</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Elena</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t>Megera</t>
-        </is>
-      </c>
-      <c r="AE36" t="inlineStr">
-        <is>
-          <t>Oste</t>
+          <t>Alessio</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Andrea</t>
+          <t>Nulter</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Andrea</t>
-        </is>
-      </c>
-      <c r="AB37" t="inlineStr">
-        <is>
-          <t>Giullare Modificato</t>
-        </is>
-      </c>
-      <c r="AD37" t="inlineStr">
-        <is>
-          <t>Oratore</t>
-        </is>
-      </c>
-      <c r="AE37" t="inlineStr">
+          <t>Nulter (MarcoC)</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AF37" t="inlineStr">
-        <is>
-          <t>Monaco</t>
-        </is>
-      </c>
-      <c r="AH37" t="inlineStr">
-        <is>
-          <t>Capobranco Maledetto</t>
-        </is>
-      </c>
       <c r="AI37" t="inlineStr">
         <is>
-          <t>Angelo</t>
+          <t>Assassino</t>
         </is>
       </c>
       <c r="AJ37" t="inlineStr">
         <is>
+          <t>Inquisitore</t>
+        </is>
+      </c>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
+      <c r="AQ37" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
+      <c r="AR37" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
+        </is>
+      </c>
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>Contadino</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+      <c r="AV37" t="inlineStr">
+        <is>
+          <t>Bracconiere</t>
+        </is>
+      </c>
+      <c r="AW37" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+      <c r="AY37" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
+      <c r="BA37" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
+      <c r="BB37" t="inlineStr">
+        <is>
           <t>Giovane Lupo</t>
         </is>
       </c>
-      <c r="AK37" t="inlineStr">
-        <is>
-          <t>Lupo Reietto</t>
-        </is>
-      </c>
-      <c r="AL37" t="inlineStr">
-        <is>
-          <t>Strega</t>
+      <c r="BC37" t="inlineStr">
+        <is>
+          <t>Capogilda</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alessio</t>
+          <t>Krobbi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alessio</t>
-        </is>
-      </c>
-      <c r="AC38" t="inlineStr">
-        <is>
-          <t>Pazzo</t>
-        </is>
-      </c>
-      <c r="AG38" t="inlineStr">
-        <is>
-          <t>Fanatico</t>
+          <t>Krobbi</t>
+        </is>
+      </c>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>Contadino</t>
+        </is>
+      </c>
+      <c r="AV38" t="inlineStr">
+        <is>
+          <t>Guaritore</t>
+        </is>
+      </c>
+      <c r="AY38" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+      <c r="AZ38" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="BB38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="BC38" t="inlineStr">
+        <is>
+          <t>Monaco</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Nulter</t>
+          <t>Garuni</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nulter (MarcoC)</t>
-        </is>
-      </c>
-      <c r="AH39" t="inlineStr">
+          <t>Garuni</t>
+        </is>
+      </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
+      <c r="BB39" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
+      <c r="BC39" t="inlineStr">
         <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="AI39" t="inlineStr">
-        <is>
-          <t>Assassino</t>
-        </is>
-      </c>
-      <c r="AJ39" t="inlineStr">
-        <is>
-          <t>Inquisitore</t>
-        </is>
-      </c>
-      <c r="AK39" t="inlineStr">
-        <is>
-          <t>Capobranco</t>
-        </is>
-      </c>
-      <c r="AN39" t="inlineStr">
-        <is>
-          <t>Eremita</t>
-        </is>
-      </c>
-      <c r="AO39" t="inlineStr">
-        <is>
-          <t>Mago</t>
-        </is>
-      </c>
-      <c r="AQ39" t="inlineStr">
-        <is>
-          <t>Lupo del Branco</t>
-        </is>
-      </c>
-      <c r="AR39" t="inlineStr">
-        <is>
-          <t>Pazzo</t>
-        </is>
-      </c>
-      <c r="AS39" t="inlineStr">
-        <is>
-          <t>Contadino</t>
-        </is>
-      </c>
-      <c r="AU39" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="AV39" t="inlineStr">
-        <is>
-          <t>Bracconiere</t>
-        </is>
-      </c>
-      <c r="AW39" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="AY39" t="inlineStr">
-        <is>
-          <t>Bardo</t>
-        </is>
-      </c>
-      <c r="BA39" t="inlineStr">
-        <is>
-          <t>Lupo del Branco</t>
-        </is>
-      </c>
-      <c r="BB39" t="inlineStr">
-        <is>
-          <t>Giovane Lupo</t>
-        </is>
-      </c>
-      <c r="BC39" t="inlineStr">
-        <is>
-          <t>Capogilda</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Krobbi</t>
+          <t>Mattia</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Krobbi</t>
-        </is>
-      </c>
-      <c r="AL40" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="AM40" t="inlineStr">
-        <is>
-          <t>Contadino</t>
-        </is>
-      </c>
-      <c r="AV40" t="inlineStr">
-        <is>
-          <t>Guaritore</t>
-        </is>
-      </c>
-      <c r="AY40" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="AZ40" t="inlineStr">
-        <is>
-          <t>Monaco</t>
-        </is>
-      </c>
-      <c r="BB40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="BC40" t="inlineStr">
-        <is>
-          <t>Monaco</t>
+          <t>Mattia</t>
+        </is>
+      </c>
+      <c r="AQ40" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
+      <c r="AR40" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>Mago</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Garuni</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Garuni</t>
-        </is>
-      </c>
-      <c r="AL41" t="inlineStr">
-        <is>
-          <t>Giullare Modificato</t>
-        </is>
-      </c>
-      <c r="AV41" t="inlineStr">
-        <is>
-          <t>Mercante</t>
-        </is>
-      </c>
-      <c r="BB41" t="inlineStr">
-        <is>
-          <t>Cacciatore di Vampiri</t>
-        </is>
-      </c>
-      <c r="BC41" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="AQ41" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
+      <c r="AR41" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>Eremita</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mattia</t>
+          <t>Vincenzo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mattia</t>
-        </is>
-      </c>
-      <c r="AQ42" t="inlineStr">
-        <is>
-          <t>Strega</t>
-        </is>
-      </c>
-      <c r="AR42" t="inlineStr">
-        <is>
-          <t>Bardo</t>
-        </is>
-      </c>
-      <c r="AS42" t="inlineStr">
+          <t>Vincenzo</t>
+        </is>
+      </c>
+      <c r="AZ42" t="inlineStr">
         <is>
           <t>Mago</t>
         </is>
@@ -6812,101 +6808,57 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Johnny</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Sergio</t>
-        </is>
-      </c>
-      <c r="AQ43" t="inlineStr">
+          <t>Giovanni</t>
+        </is>
+      </c>
+      <c r="AZ43" t="inlineStr">
         <is>
           <t>Veggente</t>
         </is>
       </c>
-      <c r="AR43" t="inlineStr">
-        <is>
-          <t>Monaco</t>
-        </is>
-      </c>
-      <c r="AS43" t="inlineStr">
-        <is>
-          <t>Eremita</t>
+      <c r="BA43" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="BB43" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="BC43" t="inlineStr">
+        <is>
+          <t>Lupo Solitario</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vincenzo</t>
+          <t>Trama</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vincenzo</t>
+          <t>Mattia</t>
         </is>
       </c>
       <c r="AZ44" t="inlineStr">
         <is>
-          <t>Mago</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Johnny</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Giovanni</t>
-        </is>
-      </c>
-      <c r="AZ45" t="inlineStr">
-        <is>
-          <t>Veggente</t>
-        </is>
-      </c>
-      <c r="BA45" t="inlineStr">
-        <is>
-          <t>Capobranco</t>
-        </is>
-      </c>
-      <c r="BB45" t="inlineStr">
-        <is>
-          <t>Capobranco</t>
-        </is>
-      </c>
-      <c r="BC45" t="inlineStr">
-        <is>
-          <t>Lupo Solitario</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Mattia Trama</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Mattia Trama</t>
-        </is>
-      </c>
-      <c r="AZ46" t="inlineStr">
-        <is>
           <t>Capobranco Maledetto</t>
         </is>
       </c>
-      <c r="BA46" t="inlineStr">
+      <c r="BA44" t="inlineStr">
         <is>
           <t>Monaco</t>
         </is>
       </c>
-      <c r="BB46" t="inlineStr">
+      <c r="BB44" t="inlineStr">
         <is>
           <t>Vampiro</t>
         </is>

</xml_diff>

<commit_message>
Rename modalita Live -> In persona Live; add 'Tutte Live' (Discord Live + In persona Live) filter
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -10394,7 +10394,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>In persona Live</t>
         </is>
       </c>
     </row>
@@ -10406,7 +10406,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>In persona Live</t>
         </is>
       </c>
     </row>
@@ -10418,7 +10418,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>In persona Live</t>
         </is>
       </c>
     </row>

</xml_diff>